<commit_message>
feat: complete donor-recipient-volunteer workflow, multi-IP support, MongoDB persistence, and mobile UI fixes
</commit_message>
<xml_diff>
--- a/backend/auth-test-results.xlsx
+++ b/backend/auth-test-results.xlsx
@@ -417,7 +417,7 @@
         <v>Generated On</v>
       </c>
       <c r="B2" t="str">
-        <v>24/7/2026, 2:51:33 pm</v>
+        <v>25/7/2026, 12:44:32 am</v>
       </c>
     </row>
     <row r="3">
@@ -473,7 +473,7 @@
         <v>Total Execution Duration</v>
       </c>
       <c r="B9" t="str">
-        <v>4.35 seconds</v>
+        <v>4.58 seconds</v>
       </c>
     </row>
   </sheetData>
@@ -550,7 +550,7 @@
         <v>PASS</v>
       </c>
       <c r="H2">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I2" t="str">
         <v>Low</v>
@@ -579,7 +579,7 @@
         <v>PASS</v>
       </c>
       <c r="H3">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="I3" t="str">
         <v>Medium</v>
@@ -608,7 +608,7 @@
         <v>PASS</v>
       </c>
       <c r="H4">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="I4" t="str">
         <v>High</v>
@@ -637,7 +637,7 @@
         <v>PASS</v>
       </c>
       <c r="H5">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="I5" t="str">
         <v>Critical</v>
@@ -666,7 +666,7 @@
         <v>PASS</v>
       </c>
       <c r="H6">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="I6" t="str">
         <v>Low</v>
@@ -695,7 +695,7 @@
         <v>PASS</v>
       </c>
       <c r="H7">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I7" t="str">
         <v>High</v>
@@ -724,7 +724,7 @@
         <v>PASS</v>
       </c>
       <c r="H8">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I8" t="str">
         <v>Low</v>
@@ -753,7 +753,7 @@
         <v>PASS</v>
       </c>
       <c r="H9">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I9" t="str">
         <v>Critical</v>
@@ -782,7 +782,7 @@
         <v>PASS</v>
       </c>
       <c r="H10">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I10" t="str">
         <v>High</v>
@@ -840,7 +840,7 @@
         <v>PASS</v>
       </c>
       <c r="H12">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I12" t="str">
         <v>Low</v>
@@ -869,7 +869,7 @@
         <v>PASS</v>
       </c>
       <c r="H13">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I13" t="str">
         <v>Medium</v>
@@ -898,7 +898,7 @@
         <v>PASS</v>
       </c>
       <c r="H14">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I14" t="str">
         <v>High</v>
@@ -927,7 +927,7 @@
         <v>PASS</v>
       </c>
       <c r="H15">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="I15" t="str">
         <v>Critical</v>
@@ -956,7 +956,7 @@
         <v>PASS</v>
       </c>
       <c r="H16">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I16" t="str">
         <v>Low</v>
@@ -985,7 +985,7 @@
         <v>PASS</v>
       </c>
       <c r="H17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I17" t="str">
         <v>High</v>
@@ -1014,7 +1014,7 @@
         <v>PASS</v>
       </c>
       <c r="H18">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="I18" t="str">
         <v>Low</v>
@@ -1043,7 +1043,7 @@
         <v>PASS</v>
       </c>
       <c r="H19">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I19" t="str">
         <v>Critical</v>
@@ -1072,7 +1072,7 @@
         <v>PASS</v>
       </c>
       <c r="H20">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="I20" t="str">
         <v>High</v>
@@ -1101,7 +1101,7 @@
         <v>PASS</v>
       </c>
       <c r="H21">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="I21" t="str">
         <v>Medium</v>
@@ -1130,7 +1130,7 @@
         <v>PASS</v>
       </c>
       <c r="H22">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I22" t="str">
         <v>Low</v>
@@ -1159,7 +1159,7 @@
         <v>PASS</v>
       </c>
       <c r="H23">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I23" t="str">
         <v>Medium</v>
@@ -1188,7 +1188,7 @@
         <v>PASS</v>
       </c>
       <c r="H24">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I24" t="str">
         <v>High</v>
@@ -1217,7 +1217,7 @@
         <v>PASS</v>
       </c>
       <c r="H25">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I25" t="str">
         <v>Critical</v>
@@ -1246,7 +1246,7 @@
         <v>PASS</v>
       </c>
       <c r="H26">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I26" t="str">
         <v>Low</v>
@@ -1275,7 +1275,7 @@
         <v>PASS</v>
       </c>
       <c r="H27">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="I27" t="str">
         <v>High</v>
@@ -1304,7 +1304,7 @@
         <v>PASS</v>
       </c>
       <c r="H28">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="I28" t="str">
         <v>Low</v>
@@ -1333,7 +1333,7 @@
         <v>PASS</v>
       </c>
       <c r="H29">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I29" t="str">
         <v>Critical</v>
@@ -1362,7 +1362,7 @@
         <v>PASS</v>
       </c>
       <c r="H30">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I30" t="str">
         <v>High</v>
@@ -1391,7 +1391,7 @@
         <v>PASS</v>
       </c>
       <c r="H31">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="I31" t="str">
         <v>Medium</v>
@@ -1420,7 +1420,7 @@
         <v>PASS</v>
       </c>
       <c r="H32">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I32" t="str">
         <v>Low</v>
@@ -1449,7 +1449,7 @@
         <v>PASS</v>
       </c>
       <c r="H33">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I33" t="str">
         <v>Medium</v>
@@ -1478,7 +1478,7 @@
         <v>PASS</v>
       </c>
       <c r="H34">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I34" t="str">
         <v>High</v>
@@ -1507,7 +1507,7 @@
         <v>PASS</v>
       </c>
       <c r="H35">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I35" t="str">
         <v>Critical</v>
@@ -1536,7 +1536,7 @@
         <v>PASS</v>
       </c>
       <c r="H36">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I36" t="str">
         <v>Low</v>
@@ -1565,7 +1565,7 @@
         <v>PASS</v>
       </c>
       <c r="H37">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="I37" t="str">
         <v>High</v>
@@ -1623,7 +1623,7 @@
         <v>PASS</v>
       </c>
       <c r="H39">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I39" t="str">
         <v>Critical</v>
@@ -1652,7 +1652,7 @@
         <v>PASS</v>
       </c>
       <c r="H40">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I40" t="str">
         <v>High</v>
@@ -1681,7 +1681,7 @@
         <v>PASS</v>
       </c>
       <c r="H41">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="I41" t="str">
         <v>Medium</v>
@@ -1710,7 +1710,7 @@
         <v>PASS</v>
       </c>
       <c r="H42">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="I42" t="str">
         <v>Low</v>
@@ -1768,7 +1768,7 @@
         <v>PASS</v>
       </c>
       <c r="H44">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="I44" t="str">
         <v>High</v>
@@ -1797,7 +1797,7 @@
         <v>PASS</v>
       </c>
       <c r="H45">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I45" t="str">
         <v>Critical</v>
@@ -1826,7 +1826,7 @@
         <v>PASS</v>
       </c>
       <c r="H46">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="I46" t="str">
         <v>Low</v>
@@ -1855,7 +1855,7 @@
         <v>PASS</v>
       </c>
       <c r="H47">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I47" t="str">
         <v>High</v>
@@ -1884,7 +1884,7 @@
         <v>PASS</v>
       </c>
       <c r="H48">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I48" t="str">
         <v>Low</v>
@@ -1913,7 +1913,7 @@
         <v>PASS</v>
       </c>
       <c r="H49">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="I49" t="str">
         <v>Critical</v>
@@ -1942,7 +1942,7 @@
         <v>PASS</v>
       </c>
       <c r="H50">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I50" t="str">
         <v>High</v>
@@ -1971,7 +1971,7 @@
         <v>PASS</v>
       </c>
       <c r="H51">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="I51" t="str">
         <v>Medium</v>
@@ -2000,7 +2000,7 @@
         <v>PASS</v>
       </c>
       <c r="H52">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="I52" t="str">
         <v>Low</v>
@@ -2029,7 +2029,7 @@
         <v>PASS</v>
       </c>
       <c r="H53">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I53" t="str">
         <v>Medium</v>
@@ -2058,7 +2058,7 @@
         <v>PASS</v>
       </c>
       <c r="H54">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I54" t="str">
         <v>High</v>
@@ -2087,7 +2087,7 @@
         <v>PASS</v>
       </c>
       <c r="H55">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="I55" t="str">
         <v>Critical</v>
@@ -2116,7 +2116,7 @@
         <v>PASS</v>
       </c>
       <c r="H56">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I56" t="str">
         <v>Low</v>
@@ -2145,7 +2145,7 @@
         <v>PASS</v>
       </c>
       <c r="H57">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="I57" t="str">
         <v>High</v>
@@ -2174,7 +2174,7 @@
         <v>PASS</v>
       </c>
       <c r="H58">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="I58" t="str">
         <v>Low</v>
@@ -2203,7 +2203,7 @@
         <v>PASS</v>
       </c>
       <c r="H59">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I59" t="str">
         <v>Critical</v>
@@ -2232,7 +2232,7 @@
         <v>PASS</v>
       </c>
       <c r="H60">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I60" t="str">
         <v>High</v>
@@ -2261,7 +2261,7 @@
         <v>PASS</v>
       </c>
       <c r="H61">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I61" t="str">
         <v>Medium</v>
@@ -2290,7 +2290,7 @@
         <v>PASS</v>
       </c>
       <c r="H62">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="I62" t="str">
         <v>Low</v>
@@ -2319,7 +2319,7 @@
         <v>PASS</v>
       </c>
       <c r="H63">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I63" t="str">
         <v>Medium</v>
@@ -2348,7 +2348,7 @@
         <v>PASS</v>
       </c>
       <c r="H64">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="I64" t="str">
         <v>High</v>
@@ -2377,7 +2377,7 @@
         <v>PASS</v>
       </c>
       <c r="H65">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I65" t="str">
         <v>Critical</v>
@@ -2406,7 +2406,7 @@
         <v>PASS</v>
       </c>
       <c r="H66">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I66" t="str">
         <v>Low</v>
@@ -2435,7 +2435,7 @@
         <v>PASS</v>
       </c>
       <c r="H67">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="I67" t="str">
         <v>High</v>
@@ -2464,7 +2464,7 @@
         <v>PASS</v>
       </c>
       <c r="H68">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I68" t="str">
         <v>Low</v>
@@ -2493,7 +2493,7 @@
         <v>PASS</v>
       </c>
       <c r="H69">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I69" t="str">
         <v>Critical</v>
@@ -2522,7 +2522,7 @@
         <v>PASS</v>
       </c>
       <c r="H70">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="I70" t="str">
         <v>High</v>
@@ -2551,7 +2551,7 @@
         <v>PASS</v>
       </c>
       <c r="H71">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I71" t="str">
         <v>Medium</v>
@@ -2580,7 +2580,7 @@
         <v>PASS</v>
       </c>
       <c r="H72">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I72" t="str">
         <v>Low</v>
@@ -2609,7 +2609,7 @@
         <v>PASS</v>
       </c>
       <c r="H73">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="I73" t="str">
         <v>Medium</v>
@@ -2638,7 +2638,7 @@
         <v>PASS</v>
       </c>
       <c r="H74">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I74" t="str">
         <v>High</v>
@@ -2667,7 +2667,7 @@
         <v>PASS</v>
       </c>
       <c r="H75">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="I75" t="str">
         <v>Critical</v>
@@ -2696,7 +2696,7 @@
         <v>PASS</v>
       </c>
       <c r="H76">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I76" t="str">
         <v>Low</v>
@@ -2725,7 +2725,7 @@
         <v>PASS</v>
       </c>
       <c r="H77">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I77" t="str">
         <v>High</v>
@@ -2754,7 +2754,7 @@
         <v>PASS</v>
       </c>
       <c r="H78">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I78" t="str">
         <v>Low</v>
@@ -2783,7 +2783,7 @@
         <v>PASS</v>
       </c>
       <c r="H79">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I79" t="str">
         <v>Critical</v>
@@ -2812,7 +2812,7 @@
         <v>PASS</v>
       </c>
       <c r="H80">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I80" t="str">
         <v>High</v>
@@ -2841,7 +2841,7 @@
         <v>PASS</v>
       </c>
       <c r="H81">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I81" t="str">
         <v>Medium</v>
@@ -2870,7 +2870,7 @@
         <v>PASS</v>
       </c>
       <c r="H82">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="I82" t="str">
         <v>Low</v>
@@ -2899,7 +2899,7 @@
         <v>PASS</v>
       </c>
       <c r="H83">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="I83" t="str">
         <v>Medium</v>
@@ -2928,7 +2928,7 @@
         <v>PASS</v>
       </c>
       <c r="H84">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I84" t="str">
         <v>High</v>
@@ -2957,7 +2957,7 @@
         <v>PASS</v>
       </c>
       <c r="H85">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="I85" t="str">
         <v>Critical</v>
@@ -2986,7 +2986,7 @@
         <v>PASS</v>
       </c>
       <c r="H86">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="I86" t="str">
         <v>Low</v>
@@ -3015,7 +3015,7 @@
         <v>PASS</v>
       </c>
       <c r="H87">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I87" t="str">
         <v>High</v>
@@ -3044,7 +3044,7 @@
         <v>PASS</v>
       </c>
       <c r="H88">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="I88" t="str">
         <v>Low</v>
@@ -3073,7 +3073,7 @@
         <v>PASS</v>
       </c>
       <c r="H89">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I89" t="str">
         <v>Critical</v>
@@ -3102,7 +3102,7 @@
         <v>PASS</v>
       </c>
       <c r="H90">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I90" t="str">
         <v>High</v>
@@ -3131,7 +3131,7 @@
         <v>PASS</v>
       </c>
       <c r="H91">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I91" t="str">
         <v>Medium</v>
@@ -3160,7 +3160,7 @@
         <v>PASS</v>
       </c>
       <c r="H92">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="I92" t="str">
         <v>Low</v>
@@ -3189,7 +3189,7 @@
         <v>PASS</v>
       </c>
       <c r="H93">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="I93" t="str">
         <v>Medium</v>
@@ -3276,7 +3276,7 @@
         <v>PASS</v>
       </c>
       <c r="H96">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="I96" t="str">
         <v>Low</v>
@@ -3305,7 +3305,7 @@
         <v>PASS</v>
       </c>
       <c r="H97">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I97" t="str">
         <v>High</v>
@@ -3334,7 +3334,7 @@
         <v>PASS</v>
       </c>
       <c r="H98">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I98" t="str">
         <v>Low</v>
@@ -3363,7 +3363,7 @@
         <v>PASS</v>
       </c>
       <c r="H99">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="I99" t="str">
         <v>Critical</v>
@@ -3392,7 +3392,7 @@
         <v>PASS</v>
       </c>
       <c r="H100">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="I100" t="str">
         <v>High</v>
@@ -3421,7 +3421,7 @@
         <v>PASS</v>
       </c>
       <c r="H101">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I101" t="str">
         <v>Medium</v>
@@ -3450,7 +3450,7 @@
         <v>PASS</v>
       </c>
       <c r="H102">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="I102" t="str">
         <v>Low</v>
@@ -3479,7 +3479,7 @@
         <v>PASS</v>
       </c>
       <c r="H103">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I103" t="str">
         <v>Medium</v>
@@ -3508,7 +3508,7 @@
         <v>PASS</v>
       </c>
       <c r="H104">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I104" t="str">
         <v>High</v>
@@ -3537,7 +3537,7 @@
         <v>PASS</v>
       </c>
       <c r="H105">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I105" t="str">
         <v>Critical</v>
@@ -3566,7 +3566,7 @@
         <v>PASS</v>
       </c>
       <c r="H106">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I106" t="str">
         <v>Low</v>
@@ -3595,7 +3595,7 @@
         <v>PASS</v>
       </c>
       <c r="H107">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I107" t="str">
         <v>High</v>
@@ -3624,7 +3624,7 @@
         <v>PASS</v>
       </c>
       <c r="H108">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="I108" t="str">
         <v>Low</v>
@@ -3653,7 +3653,7 @@
         <v>PASS</v>
       </c>
       <c r="H109">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="I109" t="str">
         <v>Critical</v>
@@ -3682,7 +3682,7 @@
         <v>PASS</v>
       </c>
       <c r="H110">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="I110" t="str">
         <v>High</v>
@@ -3711,7 +3711,7 @@
         <v>PASS</v>
       </c>
       <c r="H111">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I111" t="str">
         <v>Medium</v>
@@ -3740,7 +3740,7 @@
         <v>PASS</v>
       </c>
       <c r="H112">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I112" t="str">
         <v>Low</v>
@@ -3769,7 +3769,7 @@
         <v>PASS</v>
       </c>
       <c r="H113">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I113" t="str">
         <v>Medium</v>
@@ -3798,7 +3798,7 @@
         <v>PASS</v>
       </c>
       <c r="H114">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="I114" t="str">
         <v>High</v>
@@ -3827,7 +3827,7 @@
         <v>PASS</v>
       </c>
       <c r="H115">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="I115" t="str">
         <v>Critical</v>
@@ -3856,7 +3856,7 @@
         <v>PASS</v>
       </c>
       <c r="H116">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I116" t="str">
         <v>Low</v>
@@ -3885,7 +3885,7 @@
         <v>PASS</v>
       </c>
       <c r="H117">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="I117" t="str">
         <v>High</v>
@@ -3914,7 +3914,7 @@
         <v>PASS</v>
       </c>
       <c r="H118">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="I118" t="str">
         <v>Low</v>
@@ -3943,7 +3943,7 @@
         <v>PASS</v>
       </c>
       <c r="H119">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I119" t="str">
         <v>Critical</v>
@@ -3972,7 +3972,7 @@
         <v>PASS</v>
       </c>
       <c r="H120">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I120" t="str">
         <v>High</v>
@@ -4001,7 +4001,7 @@
         <v>PASS</v>
       </c>
       <c r="H121">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I121" t="str">
         <v>Medium</v>
@@ -4030,7 +4030,7 @@
         <v>PASS</v>
       </c>
       <c r="H122">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I122" t="str">
         <v>Low</v>
@@ -4088,7 +4088,7 @@
         <v>PASS</v>
       </c>
       <c r="H124">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="I124" t="str">
         <v>High</v>
@@ -4117,7 +4117,7 @@
         <v>PASS</v>
       </c>
       <c r="H125">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I125" t="str">
         <v>Critical</v>
@@ -4146,7 +4146,7 @@
         <v>PASS</v>
       </c>
       <c r="H126">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I126" t="str">
         <v>Low</v>
@@ -4175,7 +4175,7 @@
         <v>PASS</v>
       </c>
       <c r="H127">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I127" t="str">
         <v>High</v>
@@ -4204,7 +4204,7 @@
         <v>PASS</v>
       </c>
       <c r="H128">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="I128" t="str">
         <v>Low</v>
@@ -4233,7 +4233,7 @@
         <v>PASS</v>
       </c>
       <c r="H129">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="I129" t="str">
         <v>Critical</v>
@@ -4262,7 +4262,7 @@
         <v>PASS</v>
       </c>
       <c r="H130">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="I130" t="str">
         <v>High</v>
@@ -4291,7 +4291,7 @@
         <v>PASS</v>
       </c>
       <c r="H131">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I131" t="str">
         <v>Medium</v>
@@ -4320,7 +4320,7 @@
         <v>PASS</v>
       </c>
       <c r="H132">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="I132" t="str">
         <v>Low</v>
@@ -4349,7 +4349,7 @@
         <v>PASS</v>
       </c>
       <c r="H133">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I133" t="str">
         <v>Medium</v>
@@ -4378,7 +4378,7 @@
         <v>PASS</v>
       </c>
       <c r="H134">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I134" t="str">
         <v>High</v>
@@ -4407,7 +4407,7 @@
         <v>PASS</v>
       </c>
       <c r="H135">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I135" t="str">
         <v>Critical</v>
@@ -4436,7 +4436,7 @@
         <v>PASS</v>
       </c>
       <c r="H136">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I136" t="str">
         <v>Low</v>
@@ -4465,7 +4465,7 @@
         <v>PASS</v>
       </c>
       <c r="H137">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I137" t="str">
         <v>High</v>
@@ -4494,7 +4494,7 @@
         <v>PASS</v>
       </c>
       <c r="H138">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="I138" t="str">
         <v>Low</v>
@@ -4523,7 +4523,7 @@
         <v>PASS</v>
       </c>
       <c r="H139">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I139" t="str">
         <v>Critical</v>
@@ -4552,7 +4552,7 @@
         <v>PASS</v>
       </c>
       <c r="H140">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="I140" t="str">
         <v>High</v>
@@ -4581,7 +4581,7 @@
         <v>PASS</v>
       </c>
       <c r="H141">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I141" t="str">
         <v>Medium</v>
@@ -4610,7 +4610,7 @@
         <v>PASS</v>
       </c>
       <c r="H142">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="I142" t="str">
         <v>Low</v>
@@ -4639,7 +4639,7 @@
         <v>PASS</v>
       </c>
       <c r="H143">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="I143" t="str">
         <v>Medium</v>
@@ -4668,7 +4668,7 @@
         <v>PASS</v>
       </c>
       <c r="H144">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I144" t="str">
         <v>High</v>
@@ -4697,7 +4697,7 @@
         <v>PASS</v>
       </c>
       <c r="H145">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="I145" t="str">
         <v>Critical</v>
@@ -4726,7 +4726,7 @@
         <v>PASS</v>
       </c>
       <c r="H146">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I146" t="str">
         <v>Low</v>
@@ -4755,7 +4755,7 @@
         <v>PASS</v>
       </c>
       <c r="H147">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I147" t="str">
         <v>High</v>
@@ -4784,7 +4784,7 @@
         <v>PASS</v>
       </c>
       <c r="H148">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="I148" t="str">
         <v>Low</v>
@@ -4813,7 +4813,7 @@
         <v>PASS</v>
       </c>
       <c r="H149">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="I149" t="str">
         <v>Critical</v>
@@ -4842,7 +4842,7 @@
         <v>PASS</v>
       </c>
       <c r="H150">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I150" t="str">
         <v>High</v>
@@ -4871,7 +4871,7 @@
         <v>PASS</v>
       </c>
       <c r="H151">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="I151" t="str">
         <v>Medium</v>
@@ -4900,7 +4900,7 @@
         <v>PASS</v>
       </c>
       <c r="H152">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I152" t="str">
         <v>Low</v>
@@ -4929,7 +4929,7 @@
         <v>PASS</v>
       </c>
       <c r="H153">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="I153" t="str">
         <v>Medium</v>
@@ -4958,7 +4958,7 @@
         <v>PASS</v>
       </c>
       <c r="H154">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I154" t="str">
         <v>High</v>
@@ -4987,7 +4987,7 @@
         <v>PASS</v>
       </c>
       <c r="H155">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="I155" t="str">
         <v>Critical</v>
@@ -5016,7 +5016,7 @@
         <v>PASS</v>
       </c>
       <c r="H156">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I156" t="str">
         <v>Low</v>
@@ -5045,7 +5045,7 @@
         <v>PASS</v>
       </c>
       <c r="H157">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I157" t="str">
         <v>High</v>
@@ -5074,7 +5074,7 @@
         <v>PASS</v>
       </c>
       <c r="H158">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I158" t="str">
         <v>Low</v>
@@ -5103,7 +5103,7 @@
         <v>PASS</v>
       </c>
       <c r="H159">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I159" t="str">
         <v>Critical</v>
@@ -5132,7 +5132,7 @@
         <v>PASS</v>
       </c>
       <c r="H160">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I160" t="str">
         <v>High</v>
@@ -5161,7 +5161,7 @@
         <v>PASS</v>
       </c>
       <c r="H161">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="I161" t="str">
         <v>Medium</v>
@@ -5190,7 +5190,7 @@
         <v>PASS</v>
       </c>
       <c r="H162">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="I162" t="str">
         <v>Low</v>
@@ -5219,7 +5219,7 @@
         <v>PASS</v>
       </c>
       <c r="H163">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="I163" t="str">
         <v>Medium</v>
@@ -5248,7 +5248,7 @@
         <v>PASS</v>
       </c>
       <c r="H164">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I164" t="str">
         <v>High</v>
@@ -5277,7 +5277,7 @@
         <v>PASS</v>
       </c>
       <c r="H165">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="I165" t="str">
         <v>Critical</v>
@@ -5335,7 +5335,7 @@
         <v>PASS</v>
       </c>
       <c r="H167">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="I167" t="str">
         <v>High</v>
@@ -5364,7 +5364,7 @@
         <v>PASS</v>
       </c>
       <c r="H168">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I168" t="str">
         <v>Low</v>
@@ -5393,7 +5393,7 @@
         <v>PASS</v>
       </c>
       <c r="H169">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="I169" t="str">
         <v>Critical</v>
@@ -5451,7 +5451,7 @@
         <v>PASS</v>
       </c>
       <c r="H171">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="I171" t="str">
         <v>Medium</v>
@@ -5480,7 +5480,7 @@
         <v>PASS</v>
       </c>
       <c r="H172">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="I172" t="str">
         <v>Low</v>
@@ -5509,7 +5509,7 @@
         <v>PASS</v>
       </c>
       <c r="H173">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="I173" t="str">
         <v>Medium</v>
@@ -5538,7 +5538,7 @@
         <v>PASS</v>
       </c>
       <c r="H174">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="I174" t="str">
         <v>High</v>
@@ -5567,7 +5567,7 @@
         <v>PASS</v>
       </c>
       <c r="H175">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I175" t="str">
         <v>Critical</v>
@@ -5596,7 +5596,7 @@
         <v>PASS</v>
       </c>
       <c r="H176">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I176" t="str">
         <v>Low</v>
@@ -5625,7 +5625,7 @@
         <v>PASS</v>
       </c>
       <c r="H177">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="I177" t="str">
         <v>High</v>
@@ -5654,7 +5654,7 @@
         <v>PASS</v>
       </c>
       <c r="H178">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I178" t="str">
         <v>Low</v>
@@ -5683,7 +5683,7 @@
         <v>PASS</v>
       </c>
       <c r="H179">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="I179" t="str">
         <v>Critical</v>
@@ -5712,7 +5712,7 @@
         <v>PASS</v>
       </c>
       <c r="H180">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="I180" t="str">
         <v>High</v>
@@ -5741,7 +5741,7 @@
         <v>PASS</v>
       </c>
       <c r="H181">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="I181" t="str">
         <v>Medium</v>
@@ -5770,7 +5770,7 @@
         <v>PASS</v>
       </c>
       <c r="H182">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="I182" t="str">
         <v>Low</v>
@@ -5799,7 +5799,7 @@
         <v>PASS</v>
       </c>
       <c r="H183">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I183" t="str">
         <v>Medium</v>
@@ -5828,7 +5828,7 @@
         <v>PASS</v>
       </c>
       <c r="H184">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="I184" t="str">
         <v>High</v>
@@ -5857,7 +5857,7 @@
         <v>PASS</v>
       </c>
       <c r="H185">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="I185" t="str">
         <v>Critical</v>
@@ -5886,7 +5886,7 @@
         <v>PASS</v>
       </c>
       <c r="H186">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="I186" t="str">
         <v>Low</v>
@@ -5915,7 +5915,7 @@
         <v>PASS</v>
       </c>
       <c r="H187">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I187" t="str">
         <v>High</v>
@@ -5944,7 +5944,7 @@
         <v>PASS</v>
       </c>
       <c r="H188">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I188" t="str">
         <v>Low</v>
@@ -5973,7 +5973,7 @@
         <v>PASS</v>
       </c>
       <c r="H189">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="I189" t="str">
         <v>Critical</v>
@@ -6002,7 +6002,7 @@
         <v>PASS</v>
       </c>
       <c r="H190">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I190" t="str">
         <v>High</v>
@@ -6031,7 +6031,7 @@
         <v>PASS</v>
       </c>
       <c r="H191">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I191" t="str">
         <v>Medium</v>
@@ -6060,7 +6060,7 @@
         <v>PASS</v>
       </c>
       <c r="H192">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="I192" t="str">
         <v>Low</v>
@@ -6089,7 +6089,7 @@
         <v>PASS</v>
       </c>
       <c r="H193">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="I193" t="str">
         <v>Medium</v>
@@ -6118,7 +6118,7 @@
         <v>PASS</v>
       </c>
       <c r="H194">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I194" t="str">
         <v>High</v>
@@ -6147,7 +6147,7 @@
         <v>PASS</v>
       </c>
       <c r="H195">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I195" t="str">
         <v>Critical</v>
@@ -6176,7 +6176,7 @@
         <v>PASS</v>
       </c>
       <c r="H196">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="I196" t="str">
         <v>Low</v>
@@ -6205,7 +6205,7 @@
         <v>PASS</v>
       </c>
       <c r="H197">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="I197" t="str">
         <v>High</v>
@@ -6234,7 +6234,7 @@
         <v>PASS</v>
       </c>
       <c r="H198">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="I198" t="str">
         <v>Low</v>
@@ -6263,7 +6263,7 @@
         <v>PASS</v>
       </c>
       <c r="H199">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="I199" t="str">
         <v>Critical</v>
@@ -6292,7 +6292,7 @@
         <v>PASS</v>
       </c>
       <c r="H200">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I200" t="str">
         <v>High</v>
@@ -6321,7 +6321,7 @@
         <v>PASS</v>
       </c>
       <c r="H201">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="I201" t="str">
         <v>Medium</v>
@@ -6350,7 +6350,7 @@
         <v>PASS</v>
       </c>
       <c r="H202">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="I202" t="str">
         <v>Low</v>
@@ -6379,7 +6379,7 @@
         <v>PASS</v>
       </c>
       <c r="H203">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I203" t="str">
         <v>Medium</v>
@@ -6437,7 +6437,7 @@
         <v>PASS</v>
       </c>
       <c r="H205">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I205" t="str">
         <v>Critical</v>
@@ -6466,7 +6466,7 @@
         <v>PASS</v>
       </c>
       <c r="H206">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I206" t="str">
         <v>Low</v>
@@ -6495,7 +6495,7 @@
         <v>PASS</v>
       </c>
       <c r="H207">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I207" t="str">
         <v>High</v>
@@ -6524,7 +6524,7 @@
         <v>PASS</v>
       </c>
       <c r="H208">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I208" t="str">
         <v>Low</v>
@@ -6553,7 +6553,7 @@
         <v>PASS</v>
       </c>
       <c r="H209">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I209" t="str">
         <v>Critical</v>
@@ -6582,7 +6582,7 @@
         <v>PASS</v>
       </c>
       <c r="H210">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="I210" t="str">
         <v>High</v>
@@ -6611,7 +6611,7 @@
         <v>PASS</v>
       </c>
       <c r="H211">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I211" t="str">
         <v>Medium</v>
@@ -6640,7 +6640,7 @@
         <v>PASS</v>
       </c>
       <c r="H212">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="I212" t="str">
         <v>Low</v>
@@ -6669,7 +6669,7 @@
         <v>PASS</v>
       </c>
       <c r="H213">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I213" t="str">
         <v>Medium</v>
@@ -6698,7 +6698,7 @@
         <v>PASS</v>
       </c>
       <c r="H214">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="I214" t="str">
         <v>High</v>
@@ -6727,7 +6727,7 @@
         <v>PASS</v>
       </c>
       <c r="H215">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I215" t="str">
         <v>Critical</v>
@@ -6756,7 +6756,7 @@
         <v>PASS</v>
       </c>
       <c r="H216">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="I216" t="str">
         <v>Low</v>
@@ -6814,7 +6814,7 @@
         <v>PASS</v>
       </c>
       <c r="H218">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I218" t="str">
         <v>Low</v>
@@ -6843,7 +6843,7 @@
         <v>PASS</v>
       </c>
       <c r="H219">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="I219" t="str">
         <v>Critical</v>
@@ -6872,7 +6872,7 @@
         <v>PASS</v>
       </c>
       <c r="H220">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="I220" t="str">
         <v>High</v>
@@ -6901,7 +6901,7 @@
         <v>PASS</v>
       </c>
       <c r="H221">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I221" t="str">
         <v>Medium</v>
@@ -6959,7 +6959,7 @@
         <v>PASS</v>
       </c>
       <c r="H223">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I223" t="str">
         <v>Medium</v>
@@ -6988,7 +6988,7 @@
         <v>PASS</v>
       </c>
       <c r="H224">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="I224" t="str">
         <v>High</v>
@@ -7017,7 +7017,7 @@
         <v>PASS</v>
       </c>
       <c r="H225">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I225" t="str">
         <v>Critical</v>
@@ -7046,7 +7046,7 @@
         <v>PASS</v>
       </c>
       <c r="H226">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="I226" t="str">
         <v>Low</v>
@@ -7075,7 +7075,7 @@
         <v>PASS</v>
       </c>
       <c r="H227">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="I227" t="str">
         <v>High</v>
@@ -7104,7 +7104,7 @@
         <v>PASS</v>
       </c>
       <c r="H228">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="I228" t="str">
         <v>Low</v>
@@ -7133,7 +7133,7 @@
         <v>PASS</v>
       </c>
       <c r="H229">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="I229" t="str">
         <v>Critical</v>
@@ -7162,7 +7162,7 @@
         <v>PASS</v>
       </c>
       <c r="H230">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="I230" t="str">
         <v>High</v>
@@ -7191,7 +7191,7 @@
         <v>PASS</v>
       </c>
       <c r="H231">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I231" t="str">
         <v>Medium</v>
@@ -7220,7 +7220,7 @@
         <v>PASS</v>
       </c>
       <c r="H232">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="I232" t="str">
         <v>Low</v>
@@ -7249,7 +7249,7 @@
         <v>PASS</v>
       </c>
       <c r="H233">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="I233" t="str">
         <v>Medium</v>
@@ -7278,7 +7278,7 @@
         <v>PASS</v>
       </c>
       <c r="H234">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="I234" t="str">
         <v>High</v>
@@ -7307,7 +7307,7 @@
         <v>PASS</v>
       </c>
       <c r="H235">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="I235" t="str">
         <v>Critical</v>
@@ -7336,7 +7336,7 @@
         <v>PASS</v>
       </c>
       <c r="H236">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="I236" t="str">
         <v>Low</v>
@@ -7394,7 +7394,7 @@
         <v>PASS</v>
       </c>
       <c r="H238">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I238" t="str">
         <v>Low</v>
@@ -7423,7 +7423,7 @@
         <v>PASS</v>
       </c>
       <c r="H239">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="I239" t="str">
         <v>Critical</v>
@@ -7452,7 +7452,7 @@
         <v>PASS</v>
       </c>
       <c r="H240">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I240" t="str">
         <v>High</v>
@@ -7481,7 +7481,7 @@
         <v>PASS</v>
       </c>
       <c r="H241">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="I241" t="str">
         <v>Medium</v>
@@ -7510,7 +7510,7 @@
         <v>PASS</v>
       </c>
       <c r="H242">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="I242" t="str">
         <v>Low</v>
@@ -7539,7 +7539,7 @@
         <v>PASS</v>
       </c>
       <c r="H243">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="I243" t="str">
         <v>Medium</v>
@@ -7568,7 +7568,7 @@
         <v>PASS</v>
       </c>
       <c r="H244">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="I244" t="str">
         <v>High</v>
@@ -7597,7 +7597,7 @@
         <v>PASS</v>
       </c>
       <c r="H245">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I245" t="str">
         <v>Critical</v>
@@ -7626,7 +7626,7 @@
         <v>PASS</v>
       </c>
       <c r="H246">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="I246" t="str">
         <v>Low</v>
@@ -7655,7 +7655,7 @@
         <v>PASS</v>
       </c>
       <c r="H247">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I247" t="str">
         <v>High</v>
@@ -7684,7 +7684,7 @@
         <v>PASS</v>
       </c>
       <c r="H248">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I248" t="str">
         <v>Low</v>
@@ -7713,7 +7713,7 @@
         <v>PASS</v>
       </c>
       <c r="H249">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I249" t="str">
         <v>Critical</v>
@@ -7742,7 +7742,7 @@
         <v>PASS</v>
       </c>
       <c r="H250">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I250" t="str">
         <v>High</v>
@@ -7771,7 +7771,7 @@
         <v>PASS</v>
       </c>
       <c r="H251">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="I251" t="str">
         <v>Medium</v>
@@ -7800,7 +7800,7 @@
         <v>PASS</v>
       </c>
       <c r="H252">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I252" t="str">
         <v>Low</v>
@@ -7829,7 +7829,7 @@
         <v>PASS</v>
       </c>
       <c r="H253">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I253" t="str">
         <v>Medium</v>
@@ -7887,7 +7887,7 @@
         <v>PASS</v>
       </c>
       <c r="H255">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I255" t="str">
         <v>Critical</v>
@@ -7916,7 +7916,7 @@
         <v>PASS</v>
       </c>
       <c r="H256">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I256" t="str">
         <v>Low</v>
@@ -7945,7 +7945,7 @@
         <v>PASS</v>
       </c>
       <c r="H257">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="I257" t="str">
         <v>High</v>
@@ -7974,7 +7974,7 @@
         <v>PASS</v>
       </c>
       <c r="H258">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I258" t="str">
         <v>Low</v>
@@ -8003,7 +8003,7 @@
         <v>PASS</v>
       </c>
       <c r="H259">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="I259" t="str">
         <v>Critical</v>
@@ -8032,7 +8032,7 @@
         <v>PASS</v>
       </c>
       <c r="H260">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="I260" t="str">
         <v>High</v>
@@ -8061,7 +8061,7 @@
         <v>PASS</v>
       </c>
       <c r="H261">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I261" t="str">
         <v>Medium</v>
@@ -8090,7 +8090,7 @@
         <v>PASS</v>
       </c>
       <c r="H262">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="I262" t="str">
         <v>Low</v>
@@ -8119,7 +8119,7 @@
         <v>PASS</v>
       </c>
       <c r="H263">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I263" t="str">
         <v>Medium</v>
@@ -8148,7 +8148,7 @@
         <v>PASS</v>
       </c>
       <c r="H264">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="I264" t="str">
         <v>High</v>
@@ -8177,7 +8177,7 @@
         <v>PASS</v>
       </c>
       <c r="H265">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="I265" t="str">
         <v>Critical</v>
@@ -8206,7 +8206,7 @@
         <v>PASS</v>
       </c>
       <c r="H266">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I266" t="str">
         <v>Low</v>
@@ -8235,7 +8235,7 @@
         <v>PASS</v>
       </c>
       <c r="H267">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="I267" t="str">
         <v>High</v>
@@ -8264,7 +8264,7 @@
         <v>PASS</v>
       </c>
       <c r="H268">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="I268" t="str">
         <v>Low</v>
@@ -8293,7 +8293,7 @@
         <v>PASS</v>
       </c>
       <c r="H269">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I269" t="str">
         <v>Critical</v>
@@ -8322,7 +8322,7 @@
         <v>PASS</v>
       </c>
       <c r="H270">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="I270" t="str">
         <v>High</v>
@@ -8351,7 +8351,7 @@
         <v>PASS</v>
       </c>
       <c r="H271">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="I271" t="str">
         <v>Medium</v>
@@ -8380,7 +8380,7 @@
         <v>PASS</v>
       </c>
       <c r="H272">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="I272" t="str">
         <v>Low</v>
@@ -8409,7 +8409,7 @@
         <v>PASS</v>
       </c>
       <c r="H273">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="I273" t="str">
         <v>Medium</v>
@@ -8438,7 +8438,7 @@
         <v>PASS</v>
       </c>
       <c r="H274">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="I274" t="str">
         <v>High</v>
@@ -8467,7 +8467,7 @@
         <v>PASS</v>
       </c>
       <c r="H275">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I275" t="str">
         <v>Critical</v>
@@ -8496,7 +8496,7 @@
         <v>PASS</v>
       </c>
       <c r="H276">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I276" t="str">
         <v>Low</v>
@@ -8525,7 +8525,7 @@
         <v>PASS</v>
       </c>
       <c r="H277">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="I277" t="str">
         <v>High</v>
@@ -8554,7 +8554,7 @@
         <v>PASS</v>
       </c>
       <c r="H278">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="I278" t="str">
         <v>Low</v>
@@ -8583,7 +8583,7 @@
         <v>PASS</v>
       </c>
       <c r="H279">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="I279" t="str">
         <v>Critical</v>
@@ -8612,7 +8612,7 @@
         <v>PASS</v>
       </c>
       <c r="H280">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I280" t="str">
         <v>High</v>
@@ -8641,7 +8641,7 @@
         <v>PASS</v>
       </c>
       <c r="H281">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I281" t="str">
         <v>Medium</v>
@@ -8670,7 +8670,7 @@
         <v>PASS</v>
       </c>
       <c r="H282">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I282" t="str">
         <v>Low</v>
@@ -8699,7 +8699,7 @@
         <v>PASS</v>
       </c>
       <c r="H283">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I283" t="str">
         <v>Medium</v>
@@ -8728,7 +8728,7 @@
         <v>PASS</v>
       </c>
       <c r="H284">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I284" t="str">
         <v>High</v>
@@ -8757,7 +8757,7 @@
         <v>PASS</v>
       </c>
       <c r="H285">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="I285" t="str">
         <v>Critical</v>
@@ -8815,7 +8815,7 @@
         <v>PASS</v>
       </c>
       <c r="H287">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="I287" t="str">
         <v>High</v>
@@ -8844,7 +8844,7 @@
         <v>PASS</v>
       </c>
       <c r="H288">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I288" t="str">
         <v>Low</v>
@@ -8873,7 +8873,7 @@
         <v>PASS</v>
       </c>
       <c r="H289">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="I289" t="str">
         <v>Critical</v>
@@ -8902,7 +8902,7 @@
         <v>PASS</v>
       </c>
       <c r="H290">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I290" t="str">
         <v>High</v>
@@ -8931,7 +8931,7 @@
         <v>PASS</v>
       </c>
       <c r="H291">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="I291" t="str">
         <v>Medium</v>
@@ -8960,7 +8960,7 @@
         <v>PASS</v>
       </c>
       <c r="H292">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="I292" t="str">
         <v>Low</v>
@@ -8989,7 +8989,7 @@
         <v>PASS</v>
       </c>
       <c r="H293">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="I293" t="str">
         <v>Medium</v>
@@ -9018,7 +9018,7 @@
         <v>PASS</v>
       </c>
       <c r="H294">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I294" t="str">
         <v>High</v>
@@ -9047,7 +9047,7 @@
         <v>PASS</v>
       </c>
       <c r="H295">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I295" t="str">
         <v>Critical</v>
@@ -9076,7 +9076,7 @@
         <v>PASS</v>
       </c>
       <c r="H296">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I296" t="str">
         <v>Low</v>
@@ -9105,7 +9105,7 @@
         <v>PASS</v>
       </c>
       <c r="H297">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="I297" t="str">
         <v>High</v>
@@ -9134,7 +9134,7 @@
         <v>PASS</v>
       </c>
       <c r="H298">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="I298" t="str">
         <v>Low</v>
@@ -9163,7 +9163,7 @@
         <v>PASS</v>
       </c>
       <c r="H299">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="I299" t="str">
         <v>Critical</v>
@@ -9192,7 +9192,7 @@
         <v>PASS</v>
       </c>
       <c r="H300">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="I300" t="str">
         <v>High</v>
@@ -9221,7 +9221,7 @@
         <v>PASS</v>
       </c>
       <c r="H301">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="I301" t="str">
         <v>Medium</v>
@@ -9250,7 +9250,7 @@
         <v>PASS</v>
       </c>
       <c r="H302">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I302" t="str">
         <v>Low</v>
@@ -9279,7 +9279,7 @@
         <v>PASS</v>
       </c>
       <c r="H303">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I303" t="str">
         <v>Medium</v>
@@ -9308,7 +9308,7 @@
         <v>PASS</v>
       </c>
       <c r="H304">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="I304" t="str">
         <v>High</v>
@@ -9337,7 +9337,7 @@
         <v>PASS</v>
       </c>
       <c r="H305">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="I305" t="str">
         <v>Critical</v>
@@ -9366,7 +9366,7 @@
         <v>PASS</v>
       </c>
       <c r="H306">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I306" t="str">
         <v>Low</v>
@@ -9395,7 +9395,7 @@
         <v>PASS</v>
       </c>
       <c r="H307">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="I307" t="str">
         <v>High</v>
@@ -9424,7 +9424,7 @@
         <v>PASS</v>
       </c>
       <c r="H308">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="I308" t="str">
         <v>Low</v>
@@ -9453,7 +9453,7 @@
         <v>PASS</v>
       </c>
       <c r="H309">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I309" t="str">
         <v>Critical</v>
@@ -9482,7 +9482,7 @@
         <v>PASS</v>
       </c>
       <c r="H310">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="I310" t="str">
         <v>High</v>
@@ -9511,7 +9511,7 @@
         <v>PASS</v>
       </c>
       <c r="H311">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I311" t="str">
         <v>Medium</v>
@@ -9540,7 +9540,7 @@
         <v>PASS</v>
       </c>
       <c r="H312">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I312" t="str">
         <v>Low</v>
@@ -9598,7 +9598,7 @@
         <v>PASS</v>
       </c>
       <c r="H314">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I314" t="str">
         <v>High</v>
@@ -9627,7 +9627,7 @@
         <v>PASS</v>
       </c>
       <c r="H315">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I315" t="str">
         <v>Critical</v>
@@ -9656,7 +9656,7 @@
         <v>PASS</v>
       </c>
       <c r="H316">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I316" t="str">
         <v>Low</v>
@@ -9685,7 +9685,7 @@
         <v>PASS</v>
       </c>
       <c r="H317">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I317" t="str">
         <v>High</v>
@@ -9714,7 +9714,7 @@
         <v>PASS</v>
       </c>
       <c r="H318">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="I318" t="str">
         <v>Low</v>
@@ -9743,7 +9743,7 @@
         <v>PASS</v>
       </c>
       <c r="H319">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I319" t="str">
         <v>Critical</v>
@@ -9772,7 +9772,7 @@
         <v>PASS</v>
       </c>
       <c r="H320">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I320" t="str">
         <v>High</v>
@@ -9801,7 +9801,7 @@
         <v>PASS</v>
       </c>
       <c r="H321">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="I321" t="str">
         <v>Medium</v>
@@ -9830,7 +9830,7 @@
         <v>PASS</v>
       </c>
       <c r="H322">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I322" t="str">
         <v>Low</v>
@@ -9859,7 +9859,7 @@
         <v>PASS</v>
       </c>
       <c r="H323">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I323" t="str">
         <v>Medium</v>
@@ -9888,7 +9888,7 @@
         <v>PASS</v>
       </c>
       <c r="H324">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="I324" t="str">
         <v>High</v>
@@ -9917,7 +9917,7 @@
         <v>PASS</v>
       </c>
       <c r="H325">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="I325" t="str">
         <v>Critical</v>
@@ -9946,7 +9946,7 @@
         <v>PASS</v>
       </c>
       <c r="H326">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="I326" t="str">
         <v>Low</v>
@@ -9975,7 +9975,7 @@
         <v>PASS</v>
       </c>
       <c r="H327">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I327" t="str">
         <v>High</v>
@@ -10004,7 +10004,7 @@
         <v>PASS</v>
       </c>
       <c r="H328">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="I328" t="str">
         <v>Low</v>
@@ -10033,7 +10033,7 @@
         <v>PASS</v>
       </c>
       <c r="H329">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I329" t="str">
         <v>Critical</v>
@@ -10062,7 +10062,7 @@
         <v>PASS</v>
       </c>
       <c r="H330">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="I330" t="str">
         <v>High</v>
@@ -10091,7 +10091,7 @@
         <v>PASS</v>
       </c>
       <c r="H331">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I331" t="str">
         <v>Medium</v>
@@ -10120,7 +10120,7 @@
         <v>PASS</v>
       </c>
       <c r="H332">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="I332" t="str">
         <v>Low</v>
@@ -10149,7 +10149,7 @@
         <v>PASS</v>
       </c>
       <c r="H333">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="I333" t="str">
         <v>Medium</v>
@@ -10178,7 +10178,7 @@
         <v>PASS</v>
       </c>
       <c r="H334">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="I334" t="str">
         <v>High</v>
@@ -10207,7 +10207,7 @@
         <v>PASS</v>
       </c>
       <c r="H335">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="I335" t="str">
         <v>Critical</v>
@@ -10236,7 +10236,7 @@
         <v>PASS</v>
       </c>
       <c r="H336">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I336" t="str">
         <v>Low</v>
@@ -10294,7 +10294,7 @@
         <v>PASS</v>
       </c>
       <c r="H338">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="I338" t="str">
         <v>Low</v>
@@ -10323,7 +10323,7 @@
         <v>PASS</v>
       </c>
       <c r="H339">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="I339" t="str">
         <v>Critical</v>
@@ -10352,7 +10352,7 @@
         <v>PASS</v>
       </c>
       <c r="H340">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I340" t="str">
         <v>High</v>
@@ -10381,7 +10381,7 @@
         <v>PASS</v>
       </c>
       <c r="H341">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I341" t="str">
         <v>Medium</v>
@@ -10410,7 +10410,7 @@
         <v>PASS</v>
       </c>
       <c r="H342">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="I342" t="str">
         <v>Low</v>
@@ -10439,7 +10439,7 @@
         <v>PASS</v>
       </c>
       <c r="H343">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="I343" t="str">
         <v>Medium</v>
@@ -10468,7 +10468,7 @@
         <v>PASS</v>
       </c>
       <c r="H344">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I344" t="str">
         <v>High</v>
@@ -10497,7 +10497,7 @@
         <v>PASS</v>
       </c>
       <c r="H345">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I345" t="str">
         <v>Critical</v>
@@ -10526,7 +10526,7 @@
         <v>PASS</v>
       </c>
       <c r="H346">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="I346" t="str">
         <v>Low</v>
@@ -10555,7 +10555,7 @@
         <v>PASS</v>
       </c>
       <c r="H347">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="I347" t="str">
         <v>High</v>
@@ -10584,7 +10584,7 @@
         <v>PASS</v>
       </c>
       <c r="H348">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I348" t="str">
         <v>Low</v>
@@ -10613,7 +10613,7 @@
         <v>PASS</v>
       </c>
       <c r="H349">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I349" t="str">
         <v>Critical</v>
@@ -10642,7 +10642,7 @@
         <v>PASS</v>
       </c>
       <c r="H350">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I350" t="str">
         <v>High</v>
@@ -10671,7 +10671,7 @@
         <v>PASS</v>
       </c>
       <c r="H351">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="I351" t="str">
         <v>Medium</v>

</xml_diff>